<commit_message>
Deep-dive LA (18) and Chicago (22) rosters; national total now 52
- Add LA operators: Regency Outdoor (Sunset Strip + LAX, 300+ boards),
  Bulletin Displays (top-5 freeway), Bray Outdoor, O Media Group.
- Add Chicago operators: Image Media Outdoor, Outdoor Impact, VC Outdoor,
  GreenSigns Chicago, J&B Signs, Red Star Outdoor.
- All three Tier-1 markets now have deep local rosters (NYC 29, Chicago 22, LA 18).
- README updated with per-city depth.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169X7FqU7js4G1ZKY5WjVsV
</commit_message>
<xml_diff>
--- a/florida-billboard-scraper/data/us_top_cities_billboard_companies.xlsx
+++ b/florida-billboard-scraper/data/us_top_cities_billboard_companies.xlsx
@@ -23,10 +23,10 @@
     <sheet name="About" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Companies'!$A$4:$Q$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Companies'!$A$4:$Q$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New York'!$A$4:$Q$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Los Angeles'!$A$4:$Q$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Chicago'!$A$4:$Q$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Los Angeles'!$A$4:$Q$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Chicago'!$A$4:$Q$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Houston'!$A$4:$Q$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Phoenix'!$A$4:$Q$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Philadelphia'!$A$4:$Q$14</definedName>
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -703,7 +703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>42 companies · national operators first · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville</t>
+          <t>52 companies · national operators first · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>SignAd Outdoor Advertising</t>
+          <t>Regency Outdoor Advertising</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Texas (Houston-based) + parts of Louisiana</t>
+          <t>Los Angeles / Orange County (Sunset Strip, LAX)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Houston; San Antonio; Dallas</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -2074,23 +2074,35 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>8820 Sunset Blvd</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>West Hollywood</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr"/>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>90069</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>(310) 657-8883</t>
+        </is>
+      </c>
       <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>https://www.signad.com/</t>
+          <t>https://regencyoutdoor.com/</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
@@ -2100,17 +2112,17 @@
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Premium bulletins/spectaculars — quote only, high-end</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>Largest independently owned OOH company in Texas; 2,600+ displays.</t>
+          <t>Est. 1974; SoCal's foremost private OOH firm. 300+ billboards &amp; wallscapes, dominant Sunset Strip presence + LAX exterior. (Sold 35 Strip boards to Netflix for $150M in 2018.)</t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr">
         <is>
-          <t>signad.com; WebSearch 2026-07-08</t>
+          <t>regencyoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
@@ -2122,22 +2134,22 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>American Outdoor Advertising</t>
+          <t>SignAd Outdoor Advertising</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>Texas (Houston-based) + parts of Louisiana</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>Houston; San Antonio; Dallas</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -2146,10 +2158,14 @@
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr"/>
-      <c r="G24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr"/>
@@ -2157,7 +2173,7 @@
       <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>https://www.americanoutdoor.com/</t>
+          <t>https://www.signad.com/</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
@@ -2172,24 +2188,24 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>Digital &amp; static billboards on high-traffic San Diego routes.</t>
+          <t>Largest independently owned OOH company in Texas; 2,600+ displays.</t>
         </is>
       </c>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>americanoutdoor.com; WebSearch 2026-07-08</t>
+          <t>signad.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Arizona Billboard Company</t>
+          <t>American Outdoor Advertising</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -2199,12 +2215,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Phoenix / Arizona</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2213,14 +2229,10 @@
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr"/>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
+      <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr"/>
@@ -2228,7 +2240,7 @@
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>https://arizonabillboardcompany.com/</t>
+          <t>https://www.americanoutdoor.com/</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
@@ -2243,12 +2255,12 @@
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>30+ yrs; billboards, digital LED, buses, shelters, airports, stadiums.</t>
+          <t>Digital &amp; static billboards on high-traffic San Diego routes.</t>
         </is>
       </c>
       <c r="P25" s="5" t="inlineStr">
         <is>
-          <t>arizonabillboardcompany.com; WebSearch 2026-07-08</t>
+          <t>americanoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
@@ -2260,22 +2272,22 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>BM Outdoor Media</t>
+          <t>Arizona Billboard Company</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>44 Texas cities + Phoenix</t>
+          <t>Phoenix / Arizona</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio; Phoenix</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2284,10 +2296,14 @@
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
-      <c r="G26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr"/>
@@ -2295,7 +2311,7 @@
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://bmoutdoor.com/</t>
+          <t>https://arizonabillboardcompany.com/</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -2310,12 +2326,12 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
+          <t>30+ yrs; billboards, digital LED, buses, shelters, airports, stadiums.</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>bmoutdoor.com; WebSearch 2026-07-08</t>
+          <t>arizonabillboardcompany.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
@@ -2327,22 +2343,22 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Colossal Media</t>
+          <t>BM Outdoor Media</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>New York (Brooklyn) — hand-painted murals/wallscapes</t>
+          <t>44 Texas cities + Phoenix</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston; Dallas; San Antonio; Phoenix</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2351,14 +2367,10 @@
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>Brooklyn</t>
-        </is>
-      </c>
+      <c r="G27" s="5" t="inlineStr"/>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr"/>
@@ -2366,7 +2378,7 @@
       <c r="K27" s="5" t="inlineStr"/>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://colossalmedia.com/</t>
+          <t>https://bmoutdoor.com/</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2376,17 +2388,17 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Hand-painted wallscape / mural — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t>Specialist in hand-painted outdoor advertising &amp; public-art wallscapes.</t>
+          <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
         </is>
       </c>
       <c r="P27" s="5" t="inlineStr">
         <is>
-          <t>colossalmedia.com; WebSearch 2026-07-08</t>
+          <t>bmoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
@@ -2398,7 +2410,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Gilbreath Outdoor Advertising</t>
+          <t>Bulletin Displays</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -2408,12 +2420,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Greater Houston + Texas Hill Country</t>
+          <t>Los Angeles (freeway billboards)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Houston; San Antonio</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2424,12 +2436,12 @@
       <c r="F28" s="5" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
@@ -2437,7 +2449,7 @@
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://www.gilbreathoutdoor.com/</t>
+          <t>https://www.bulletindisplays.com/</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
@@ -2452,12 +2464,12 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>Houston-area operator with a Texas Hill Country satellite office.</t>
+          <t>One of the top-5 freeway billboard operators in the LA area; digital &amp; static.</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>gilbreathoutdoor.com; WebSearch 2026-07-08</t>
+          <t>bulletindisplays.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
@@ -2469,17 +2481,17 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>InSite Street Media</t>
+          <t>Colossal Media</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>New York DMA (top-5 by spot count)</t>
+          <t>New York (Brooklyn) — hand-painted murals/wallscapes</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2495,7 +2507,7 @@
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2508,7 +2520,7 @@
       <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://www.insitestreetmedia.com/</t>
+          <t>https://colossalmedia.com/</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
@@ -2518,17 +2530,17 @@
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Hand-painted wallscape / mural — quote only</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>Top-5 NYC DMA operator; residential &amp; street-level media networks.</t>
+          <t>Specialist in hand-painted outdoor advertising &amp; public-art wallscapes.</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>oohtoday.com Top-5 NYC operators; WebSearch 2026-07-08</t>
+          <t>colossalmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
@@ -2540,22 +2552,22 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Lux Media</t>
+          <t>Gilbreath Outdoor Advertising</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Dallas; Houston; Austin; San Antonio</t>
+          <t>Greater Houston + Texas Hill Country</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Houston; San Antonio; Dallas</t>
+          <t>Houston; San Antonio</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2564,10 +2576,14 @@
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr"/>
@@ -2575,7 +2591,7 @@
       <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>https://www.luxmediaads.com/</t>
+          <t>https://www.gilbreathoutdoor.com/</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -2585,17 +2601,17 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — day/route rate, quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED billboard truck advertising across major TX metros.</t>
+          <t>Houston-area operator with a Texas Hill Country satellite office.</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>luxmediaads.com; WebSearch 2026-07-08</t>
+          <t>gilbreathoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -2607,7 +2623,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>MediaLease OOH — Jacksonville</t>
+          <t>Image Media Outdoor</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -2617,12 +2633,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2631,10 +2647,14 @@
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr"/>
@@ -2642,7 +2662,7 @@
       <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>https://www.medialeaseooh.com/jacksonville-fl/</t>
+          <t>https://imageoutdoor.com/</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
@@ -2657,12 +2677,12 @@
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>Digital LED + traditional billboards, bus, rail, shelter ads in Jacksonville.</t>
+          <t>Billboard, bulletin, digital &amp; wall advertising across Chicagoland.</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>medialeaseooh.com; WebSearch 2026-07-08</t>
+          <t>imageoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
@@ -2674,7 +2694,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>PMD Media</t>
+          <t>InSite Street Media</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -2711,7 +2731,11 @@
       <c r="I32" s="5" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="5" t="inlineStr"/>
-      <c r="L32" s="5" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.insitestreetmedia.com/</t>
+        </is>
+      </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2724,7 +2748,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Among the top-5 OOH owners in the NYC DMA by spot count.</t>
+          <t>Top-5 NYC DMA operator; residential &amp; street-level media networks.</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
@@ -2741,22 +2765,22 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>SILVERCAST Media</t>
+          <t>Lux Media</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>New York (spectaculars: Times Sq, Penn Plaza, MSG)</t>
+          <t>Dallas; Houston; Austin; San Antonio</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston; San Antonio; Dallas</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2765,14 +2789,10 @@
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr"/>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -2780,7 +2800,7 @@
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.silvercastmedia.com/</t>
+          <t>https://www.luxmediaads.com/</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
@@ -2790,17 +2810,17 @@
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Oversized digital/static spectaculars — quote only, high-end</t>
+          <t>Mobile LED truck — day/route rate, quote only</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>Premier oversized billboard spectaculars at Times Sq, Penn Plaza &amp; Madison Square Garden.</t>
+          <t>Mobile LED billboard truck advertising across major TX metros.</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr">
         <is>
-          <t>silvercastmedia.com; WebSearch 2026-07-08</t>
+          <t>luxmediaads.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q33" s="5" t="inlineStr">
@@ -2812,7 +2832,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Adams Outdoor Advertising</t>
+          <t>MediaLease OOH — Jacksonville</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -2822,12 +2842,12 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>New York DMA + mid-size US markets</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2845,7 +2865,11 @@
       <c r="I34" s="5" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr"/>
       <c r="K34" s="5" t="inlineStr"/>
-      <c r="L34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.medialeaseooh.com/jacksonville-fl/</t>
+        </is>
+      </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2858,24 +2882,24 @@
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>Traditional + digital billboards in high-visibility locations.</t>
+          <t>Digital LED + traditional billboards, bus, rail, shelter ads in Jacksonville.</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>medialeaseooh.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q34" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Big Outdoor</t>
+          <t>Outdoor Impact</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -2885,12 +2909,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>New York (digital spectaculars)</t>
+          <t>Chicago (north side)</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2901,12 +2925,12 @@
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -2914,7 +2938,7 @@
       <c r="K35" s="5" t="inlineStr"/>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://bigoutdoor.com/</t>
+          <t>https://www.outdoorimpact.com/</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -2924,44 +2948,44 @@
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Digital spectacular — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>NYC digital billboard / spectacular operator.</t>
+          <t>Billboard &amp; wall-display advertising, esp. northern Chicago.</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>outdoorimpact.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q35" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Billboards America</t>
+          <t>PMD Media</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
+          <t>New York DMA (top-5 by spot count)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2970,20 +2994,20 @@
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr"/>
-      <c r="G36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr"/>
       <c r="K36" s="5" t="inlineStr"/>
-      <c r="L36" s="5" t="inlineStr">
-        <is>
-          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
-        </is>
-      </c>
+      <c r="L36" s="5" t="inlineStr"/>
       <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2996,24 +3020,24 @@
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>Brokerage with access to prime TX billboard locations.</t>
+          <t>Among the top-5 OOH owners in the NYC DMA by spot count.</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr">
         <is>
-          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
+          <t>oohtoday.com Top-5 NYC operators; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>GSB Digital</t>
+          <t>SILVERCAST Media</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -3023,7 +3047,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>New York — wildposting / wheatpaste, print &amp; install</t>
+          <t>New York (spectaculars: Times Sq, Penn Plaza, MSG)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -3052,7 +3076,7 @@
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>https://gsbdigital.com/</t>
+          <t>https://www.silvercastmedia.com/</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
@@ -3062,39 +3086,39 @@
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Wildposting / production — quote only</t>
+          <t>Oversized digital/static spectaculars — quote only, high-end</t>
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
+          <t>Premier oversized billboard spectaculars at Times Sq, Penn Plaza &amp; Madison Square Garden.</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr">
         <is>
-          <t>gsbdigital.com; WebSearch 2026-07-08</t>
+          <t>silvercastmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q37" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Heritage Outdoor Media</t>
+          <t>Adams Outdoor Advertising</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>New York (Times Square digital)</t>
+          <t>New York DMA + mid-size US markets</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -3108,14 +3132,10 @@
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr"/>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G38" s="5" t="inlineStr"/>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr"/>
@@ -3129,12 +3149,12 @@
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Times Square digital — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Times Square LED billboard technology.</t>
+          <t>Traditional + digital billboards in high-visibility locations.</t>
         </is>
       </c>
       <c r="P38" s="5" t="inlineStr">
@@ -3151,7 +3171,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>MH Outdoor Media</t>
+          <t>Big Outdoor</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -3161,12 +3181,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>New York (digital spectaculars)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -3177,18 +3197,22 @@
       <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr"/>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="inlineStr"/>
-      <c r="L39" s="5" t="inlineStr"/>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>https://bigoutdoor.com/</t>
+        </is>
+      </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3196,12 +3220,12 @@
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Digital spectacular — quote only</t>
         </is>
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>Local Houston billboard operator.</t>
+          <t>NYC digital billboard / spectacular operator.</t>
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr">
@@ -3218,22 +3242,22 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Neutron Media</t>
+          <t>Billboards America</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>New York (digital billboards)</t>
+          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston; Dallas; San Antonio</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3242,20 +3266,20 @@
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr"/>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G40" s="5" t="inlineStr"/>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr"/>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="inlineStr"/>
-      <c r="L40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
+        </is>
+      </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3268,12 +3292,12 @@
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>Digital billboards in NYC's busiest corridors.</t>
+          <t>Brokerage with access to prime TX billboard locations.</t>
         </is>
       </c>
       <c r="P40" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
@@ -3285,22 +3309,22 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Pearl Media</t>
+          <t>Bray Outdoor Ads</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>New York / Times Square + experiential</t>
+          <t>Los Angeles County</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3309,14 +3333,10 @@
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr"/>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G41" s="5" t="inlineStr"/>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr"/>
@@ -3324,7 +3344,7 @@
       <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://pearlmedia.com/</t>
+          <t>https://brayoutdoor.com/los-angeles-county/los-angeles-billboards/</t>
         </is>
       </c>
       <c r="M41" s="5" t="inlineStr">
@@ -3334,17 +3354,17 @@
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Times Square / experiential — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>Times Square billboards and experiential activations.</t>
+          <t>LA-county billboard operator/agency.</t>
         </is>
       </c>
       <c r="P41" s="5" t="inlineStr">
         <is>
-          <t>pearlmedia.com; WebSearch 2026-07-08</t>
+          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q41" s="5" t="inlineStr">
@@ -3356,22 +3376,22 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Premier Mobile Billboards</t>
+          <t>GreenSigns Chicago</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>Chicago (all-digital network)</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -3382,22 +3402,18 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr"/>
       <c r="J42" s="5" t="inlineStr"/>
       <c r="K42" s="5" t="inlineStr"/>
-      <c r="L42" s="5" t="inlineStr">
-        <is>
-          <t>https://premiermobilebillboards.com/houston/</t>
-        </is>
-      </c>
+      <c r="L42" s="5" t="inlineStr"/>
       <c r="M42" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3405,17 +3421,17 @@
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — quote only</t>
+          <t>Digital billboard — quote only</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>Digital billboard trucks; Houston + Woodlands, Sugar Land, Katy.</t>
+          <t>Fully digital, eco-friendly billboard network.</t>
         </is>
       </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q42" s="5" t="inlineStr">
@@ -3427,7 +3443,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Red Rock Outdoor Advertising</t>
+          <t>GSB Digital</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -3437,7 +3453,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>New York (Manhattan)</t>
+          <t>New York — wildposting / wheatpaste, print &amp; install</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -3464,7 +3480,11 @@
       <c r="I43" s="5" t="inlineStr"/>
       <c r="J43" s="5" t="inlineStr"/>
       <c r="K43" s="5" t="inlineStr"/>
-      <c r="L43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>https://gsbdigital.com/</t>
+        </is>
+      </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3472,17 +3492,17 @@
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Wildposting / production — quote only</t>
         </is>
       </c>
       <c r="O43" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
         </is>
       </c>
       <c r="P43" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>gsbdigital.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q43" s="5" t="inlineStr">
@@ -3494,17 +3514,17 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Rolling Adz Mobile Billboards</t>
+          <t>Heritage Outdoor Media</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>New York City (mobile)</t>
+          <t>New York (Times Square digital)</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -3531,11 +3551,7 @@
       <c r="I44" s="5" t="inlineStr"/>
       <c r="J44" s="5" t="inlineStr"/>
       <c r="K44" s="5" t="inlineStr"/>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>https://rollingadz.com/</t>
-        </is>
-      </c>
+      <c r="L44" s="5" t="inlineStr"/>
       <c r="M44" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3543,17 +3559,17 @@
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard — day/route rate, quote only</t>
+          <t>Times Square digital — quote only</t>
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard fleet across NYC.</t>
+          <t>Times Square LED billboard technology.</t>
         </is>
       </c>
       <c r="P44" s="5" t="inlineStr">
         <is>
-          <t>rollingadz.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q44" s="5" t="inlineStr">
@@ -3565,7 +3581,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Seen Outdoor Media, LLC</t>
+          <t>J&amp;B Signs Inc</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -3575,12 +3591,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>New York (Brooklyn)</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3591,12 +3607,12 @@
       <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr"/>
@@ -3615,12 +3631,12 @@
       </c>
       <c r="O45" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Independent OOH media company partnering with local/regional/national advertisers.</t>
         </is>
       </c>
       <c r="P45" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q45" s="5" t="inlineStr">
@@ -3632,7 +3648,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>TSX Broadway (TSX Entertainment)</t>
+          <t>MH Outdoor Media</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -3642,12 +3658,12 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Times Square (single landmark asset)</t>
+          <t>Houston metro</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3658,12 +3674,12 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr"/>
@@ -3677,27 +3693,709 @@
       </c>
       <c r="N46" s="5" t="inlineStr">
         <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>Local Houston billboard operator.</t>
+        </is>
+      </c>
+      <c r="P46" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Neutron Media</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>New York (digital billboards)</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr"/>
+      <c r="J47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr"/>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O47" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboards in NYC's busiest corridors.</t>
+        </is>
+      </c>
+      <c r="P47" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>O Media Group</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O48" s="5" t="inlineStr">
+        <is>
+          <t>LA independent OOH operator (named among Regency's LA competitors).</t>
+        </is>
+      </c>
+      <c r="P48" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Pearl Media</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>New York / Times Square + experiential</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="inlineStr"/>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>https://pearlmedia.com/</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>Times Square / experiential — quote only</t>
+        </is>
+      </c>
+      <c r="O49" s="5" t="inlineStr">
+        <is>
+          <t>Times Square billboards and experiential activations.</t>
+        </is>
+      </c>
+      <c r="P49" s="5" t="inlineStr">
+        <is>
+          <t>pearlmedia.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Premier Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Houston metro</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr"/>
+      <c r="J50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="inlineStr"/>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>https://premiermobilebillboards.com/houston/</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — quote only</t>
+        </is>
+      </c>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboard trucks; Houston + Woodlands, Sugar Land, Katy.</t>
+        </is>
+      </c>
+      <c r="P50" s="5" t="inlineStr">
+        <is>
+          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Red Rock Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>New York (Manhattan)</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
+      <c r="J51" s="5" t="inlineStr"/>
+      <c r="K51" s="5" t="inlineStr"/>
+      <c r="L51" s="5" t="inlineStr"/>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O51" s="5" t="inlineStr">
+        <is>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+        </is>
+      </c>
+      <c r="P51" s="5" t="inlineStr">
+        <is>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Red Star Outdoor</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr"/>
+      <c r="K52" s="5" t="inlineStr"/>
+      <c r="L52" s="5" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O52" s="5" t="inlineStr">
+        <is>
+          <t>Chicago-market billboard operator (named among major Chicago operators).</t>
+        </is>
+      </c>
+      <c r="P52" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Rolling Adz Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>New York City (mobile)</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr"/>
+      <c r="J53" s="5" t="inlineStr"/>
+      <c r="K53" s="5" t="inlineStr"/>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>https://rollingadz.com/</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard — day/route rate, quote only</t>
+        </is>
+      </c>
+      <c r="O53" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard fleet across NYC.</t>
+        </is>
+      </c>
+      <c r="P53" s="5" t="inlineStr">
+        <is>
+          <t>rollingadz.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Seen Outdoor Media, LLC</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>New York (Brooklyn)</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr"/>
+      <c r="K54" s="5" t="inlineStr"/>
+      <c r="L54" s="5" t="inlineStr"/>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O54" s="5" t="inlineStr">
+        <is>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+        </is>
+      </c>
+      <c r="P54" s="5" t="inlineStr">
+        <is>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>TSX Broadway (TSX Entertainment)</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Times Square (single landmark asset)</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr"/>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr"/>
+      <c r="J55" s="5" t="inlineStr"/>
+      <c r="K55" s="5" t="inlineStr"/>
+      <c r="L55" s="5" t="inlineStr"/>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N55" s="5" t="inlineStr">
+        <is>
           <t>Premium spectacular — quote only, very high-end</t>
         </is>
       </c>
-      <c r="O46" s="5" t="inlineStr">
+      <c r="O55" s="5" t="inlineStr">
         <is>
           <t>Flagship 18k-sq-ft curved LED at 47th &amp; Broadway, Times Square.</t>
         </is>
       </c>
-      <c r="P46" s="5" t="inlineStr">
+      <c r="P55" s="5" t="inlineStr">
         <is>
           <t>WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q46" s="5" t="inlineStr">
+      <c r="Q55" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>VC Outdoor</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Chicago (40 neighborhoods)</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr"/>
+      <c r="J56" s="5" t="inlineStr"/>
+      <c r="K56" s="5" t="inlineStr"/>
+      <c r="L56" s="5" t="inlineStr"/>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N56" s="5" t="inlineStr">
+        <is>
+          <t>Wildposting / wallscape / bus wrap — quote only</t>
+        </is>
+      </c>
+      <c r="O56" s="5" t="inlineStr">
+        <is>
+          <t>Hotspots, wild postings, wallscapes, bus wraps &amp; street furniture across 40 Chicago neighborhoods.</t>
+        </is>
+      </c>
+      <c r="P56" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q46"/>
+  <autoFilter ref="A4:Q56"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -6387,7 +7085,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Generated by fbscraper v1.0 · 42 companies · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville.</t>
+          <t>Generated by fbscraper v1.0 · 52 companies · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville.</t>
         </is>
       </c>
     </row>
@@ -9058,7 +9756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9090,7 +9788,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>14 companies serving Los Angeles · prices quote-only</t>
+          <t>18 companies serving Los Angeles · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -10155,8 +10853,296 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Regency Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles / Orange County (Sunset Strip, LAX)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>8820 Sunset Blvd</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>West Hollywood</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>90069</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>(310) 657-8883</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>https://regencyoutdoor.com/</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Premium bulletins/spectaculars — quote only, high-end</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Est. 1974; SoCal's foremost private OOH firm. 300+ billboards &amp; wallscapes, dominant Sunset Strip presence + LAX exterior. (Sold 35 Strip boards to Netflix for $150M in 2018.)</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>regencyoutdoor.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Bulletin Displays</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles (freeway billboards)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bulletindisplays.com/</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>One of the top-5 freeway billboard operators in the LA area; digital &amp; static.</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>bulletindisplays.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Bray Outdoor Ads</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles County</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>https://brayoutdoor.com/los-angeles-county/los-angeles-billboards/</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>LA-county billboard operator/agency.</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>O Media Group</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>LA independent OOH operator (named among Regency's LA competitors).</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q18"/>
+  <autoFilter ref="A4:Q22"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -10171,7 +11157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10203,7 +11189,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>16 companies serving Chicago · prices quote-only</t>
+          <t>22 companies serving Chicago · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -11410,8 +12396,418 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Image Media Outdoor</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Chicagoland</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>https://imageoutdoor.com/</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Billboard, bulletin, digital &amp; wall advertising across Chicagoland.</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>imageoutdoor.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Outdoor Impact</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Chicago (north side)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.outdoorimpact.com/</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Billboard &amp; wall-display advertising, esp. northern Chicago.</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>outdoorimpact.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>GreenSigns Chicago</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Chicago (all-digital network)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr"/>
+      <c r="K23" s="5" t="inlineStr"/>
+      <c r="L23" s="5" t="inlineStr"/>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboard — quote only</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>Fully digital, eco-friendly billboard network.</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>J&amp;B Signs Inc</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="inlineStr"/>
+      <c r="L24" s="5" t="inlineStr"/>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Independent OOH media company partnering with local/regional/national advertisers.</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Red Star Outdoor</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr"/>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>Chicago-market billboard operator (named among major Chicago operators).</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>VC Outdoor</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Chicago (40 neighborhoods)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr"/>
+      <c r="K26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr"/>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Wildposting / wallscape / bus wrap — quote only</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>Hotspots, wild postings, wallscapes, bus wraps &amp; street furniture across 40 Chicago neighborhoods.</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q20"/>
+  <autoFilter ref="A4:Q26"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>

</xml_diff>

<commit_message>
Deep-dive Texas trio: Dallas (16), Houston (16), San Antonio (14); total 59
- Dallas: add Arrington Outdoor (largest DFW independent), Ralston, Albert,
  Dallas Billboards LLC.
- Houston: add Avail Media Group, Inspiria Outdoor Advertising.
- San Antonio: add True Impact Media.
- Broaden Premier Mobile Billboards coverage to Houston/Dallas/San Antonio.
- National total now 59 companies. README updated with Texas depth.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169X7FqU7js4G1ZKY5WjVsV
</commit_message>
<xml_diff>
--- a/florida-billboard-scraper/data/us_top_cities_billboard_companies.xlsx
+++ b/florida-billboard-scraper/data/us_top_cities_billboard_companies.xlsx
@@ -23,16 +23,16 @@
     <sheet name="About" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Companies'!$A$4:$Q$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Companies'!$A$4:$Q$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New York'!$A$4:$Q$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Los Angeles'!$A$4:$Q$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Chicago'!$A$4:$Q$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Houston'!$A$4:$Q$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Houston'!$A$4:$Q$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Phoenix'!$A$4:$Q$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Philadelphia'!$A$4:$Q$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'San Antonio'!$A$4:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'San Antonio'!$A$4:$Q$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'San Diego'!$A$4:$Q$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Dallas'!$A$4:$Q$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Dallas'!$A$4:$Q$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Jacksonville'!$A$4:$Q$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q56"/>
+  <dimension ref="A1:Q63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -703,7 +703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>52 companies · national operators first · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville</t>
+          <t>59 companies · national operators first · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>BM Outdoor Media</t>
+          <t>Arrington Outdoor Advertising</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -2353,12 +2353,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>44 Texas cities + Phoenix</t>
+          <t>Dallas–Fort Worth Metroplex</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio; Phoenix</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2367,10 +2367,14 @@
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
-      <c r="G27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr"/>
@@ -2378,7 +2382,7 @@
       <c r="K27" s="5" t="inlineStr"/>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://bmoutdoor.com/</t>
+          <t>https://www.arringtonoutdoor.com/</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2393,12 +2397,12 @@
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
+          <t>Largest independent billboard company in the DFW area; bulletins &amp; digital.</t>
         </is>
       </c>
       <c r="P27" s="5" t="inlineStr">
         <is>
-          <t>bmoutdoor.com; WebSearch 2026-07-08</t>
+          <t>arringtonoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
@@ -2410,7 +2414,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Bulletin Displays</t>
+          <t>BM Outdoor Media</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -2420,12 +2424,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles (freeway billboards)</t>
+          <t>44 Texas cities + Phoenix</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston; Dallas; San Antonio; Phoenix</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2434,14 +2438,10 @@
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>Los Angeles</t>
-        </is>
-      </c>
+      <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
@@ -2449,7 +2449,7 @@
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://www.bulletindisplays.com/</t>
+          <t>https://bmoutdoor.com/</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>One of the top-5 freeway billboard operators in the LA area; digital &amp; static.</t>
+          <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>bulletindisplays.com; WebSearch 2026-07-08</t>
+          <t>bmoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
@@ -2481,22 +2481,22 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Colossal Media</t>
+          <t>Bulletin Displays</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>New York (Brooklyn) — hand-painted murals/wallscapes</t>
+          <t>Los Angeles (freeway billboards)</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2507,12 +2507,12 @@
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr"/>
@@ -2520,7 +2520,7 @@
       <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://colossalmedia.com/</t>
+          <t>https://www.bulletindisplays.com/</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
@@ -2530,17 +2530,17 @@
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Hand-painted wallscape / mural — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>Specialist in hand-painted outdoor advertising &amp; public-art wallscapes.</t>
+          <t>One of the top-5 freeway billboard operators in the LA area; digital &amp; static.</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>colossalmedia.com; WebSearch 2026-07-08</t>
+          <t>bulletindisplays.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
@@ -2552,22 +2552,22 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Gilbreath Outdoor Advertising</t>
+          <t>Colossal Media</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Greater Houston + Texas Hill Country</t>
+          <t>New York (Brooklyn) — hand-painted murals/wallscapes</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Houston; San Antonio</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2578,12 +2578,12 @@
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr"/>
@@ -2591,7 +2591,7 @@
       <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>https://www.gilbreathoutdoor.com/</t>
+          <t>https://colossalmedia.com/</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Hand-painted wallscape / mural — quote only</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>Houston-area operator with a Texas Hill Country satellite office.</t>
+          <t>Specialist in hand-painted outdoor advertising &amp; public-art wallscapes.</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>gilbreathoutdoor.com; WebSearch 2026-07-08</t>
+          <t>colossalmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -2623,7 +2623,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Image Media Outdoor</t>
+          <t>Gilbreath Outdoor Advertising</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -2633,12 +2633,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Chicagoland</t>
+          <t>Greater Houston + Texas Hill Country</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston; San Antonio</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2649,12 +2649,12 @@
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr"/>
@@ -2662,7 +2662,7 @@
       <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>https://imageoutdoor.com/</t>
+          <t>https://www.gilbreathoutdoor.com/</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
@@ -2677,12 +2677,12 @@
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>Billboard, bulletin, digital &amp; wall advertising across Chicagoland.</t>
+          <t>Houston-area operator with a Texas Hill Country satellite office.</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>imageoutdoor.com; WebSearch 2026-07-08</t>
+          <t>gilbreathoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
@@ -2694,7 +2694,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>InSite Street Media</t>
+          <t>Image Media Outdoor</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -2704,12 +2704,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>New York DMA (top-5 by spot count)</t>
+          <t>Chicagoland</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2720,12 +2720,12 @@
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr"/>
@@ -2733,7 +2733,7 @@
       <c r="K32" s="5" t="inlineStr"/>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>https://www.insitestreetmedia.com/</t>
+          <t>https://imageoutdoor.com/</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
@@ -2748,12 +2748,12 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Top-5 NYC DMA operator; residential &amp; street-level media networks.</t>
+          <t>Billboard, bulletin, digital &amp; wall advertising across Chicagoland.</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>oohtoday.com Top-5 NYC operators; WebSearch 2026-07-08</t>
+          <t>imageoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
@@ -2765,22 +2765,22 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Lux Media</t>
+          <t>InSite Street Media</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Dallas; Houston; Austin; San Antonio</t>
+          <t>New York DMA (top-5 by spot count)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Houston; San Antonio; Dallas</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2789,10 +2789,14 @@
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr"/>
-      <c r="G33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -2800,7 +2804,7 @@
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.luxmediaads.com/</t>
+          <t>https://www.insitestreetmedia.com/</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
@@ -2810,17 +2814,17 @@
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — day/route rate, quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED billboard truck advertising across major TX metros.</t>
+          <t>Top-5 NYC DMA operator; residential &amp; street-level media networks.</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr">
         <is>
-          <t>luxmediaads.com; WebSearch 2026-07-08</t>
+          <t>oohtoday.com Top-5 NYC operators; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q33" s="5" t="inlineStr">
@@ -2832,22 +2836,22 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>MediaLease OOH — Jacksonville</t>
+          <t>Lux Media</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Dallas; Houston; Austin; San Antonio</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Houston; San Antonio; Dallas</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2867,7 +2871,7 @@
       <c r="K34" s="5" t="inlineStr"/>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.medialeaseooh.com/jacksonville-fl/</t>
+          <t>https://www.luxmediaads.com/</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
@@ -2877,17 +2881,17 @@
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Mobile LED truck — day/route rate, quote only</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>Digital LED + traditional billboards, bus, rail, shelter ads in Jacksonville.</t>
+          <t>Mobile LED billboard truck advertising across major TX metros.</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr">
         <is>
-          <t>medialeaseooh.com; WebSearch 2026-07-08</t>
+          <t>luxmediaads.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q34" s="5" t="inlineStr">
@@ -2899,22 +2903,22 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Outdoor Impact</t>
+          <t>MediaLease OOH — Jacksonville</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Chicago (north side)</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2923,14 +2927,10 @@
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr"/>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
+      <c r="G35" s="5" t="inlineStr"/>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -2938,7 +2938,7 @@
       <c r="K35" s="5" t="inlineStr"/>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://www.outdoorimpact.com/</t>
+          <t>https://www.medialeaseooh.com/jacksonville-fl/</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -2953,12 +2953,12 @@
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
-          <t>Billboard &amp; wall-display advertising, esp. northern Chicago.</t>
+          <t>Digital LED + traditional billboards, bus, rail, shelter ads in Jacksonville.</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">
         <is>
-          <t>outdoorimpact.com; WebSearch 2026-07-08</t>
+          <t>medialeaseooh.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q35" s="5" t="inlineStr">
@@ -2970,22 +2970,22 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>PMD Media</t>
+          <t>Outdoor Impact</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>New York DMA (top-5 by spot count)</t>
+          <t>Chicago (north side)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2996,18 +2996,22 @@
       <c r="F36" s="5" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr"/>
       <c r="K36" s="5" t="inlineStr"/>
-      <c r="L36" s="5" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.outdoorimpact.com/</t>
+        </is>
+      </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3020,12 +3024,12 @@
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>Among the top-5 OOH owners in the NYC DMA by spot count.</t>
+          <t>Billboard &amp; wall-display advertising, esp. northern Chicago.</t>
         </is>
       </c>
       <c r="P36" s="5" t="inlineStr">
         <is>
-          <t>oohtoday.com Top-5 NYC operators; WebSearch 2026-07-08</t>
+          <t>outdoorimpact.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q36" s="5" t="inlineStr">
@@ -3037,17 +3041,17 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>SILVERCAST Media</t>
+          <t>PMD Media</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>New York (spectaculars: Times Sq, Penn Plaza, MSG)</t>
+          <t>New York DMA (top-5 by spot count)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -3074,11 +3078,7 @@
       <c r="I37" s="5" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr"/>
       <c r="K37" s="5" t="inlineStr"/>
-      <c r="L37" s="5" t="inlineStr">
-        <is>
-          <t>https://www.silvercastmedia.com/</t>
-        </is>
-      </c>
+      <c r="L37" s="5" t="inlineStr"/>
       <c r="M37" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3086,17 +3086,17 @@
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Oversized digital/static spectaculars — quote only, high-end</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
-          <t>Premier oversized billboard spectaculars at Times Sq, Penn Plaza &amp; Madison Square Garden.</t>
+          <t>Among the top-5 OOH owners in the NYC DMA by spot count.</t>
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr">
         <is>
-          <t>silvercastmedia.com; WebSearch 2026-07-08</t>
+          <t>oohtoday.com Top-5 NYC operators; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q37" s="5" t="inlineStr">
@@ -3108,17 +3108,17 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Adams Outdoor Advertising</t>
+          <t>SILVERCAST Media</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>New York DMA + mid-size US markets</t>
+          <t>New York (spectaculars: Times Sq, Penn Plaza, MSG)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -3132,16 +3132,24 @@
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr"/>
-      <c r="G38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr"/>
       <c r="K38" s="5" t="inlineStr"/>
-      <c r="L38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.silvercastmedia.com/</t>
+        </is>
+      </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3149,39 +3157,39 @@
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Oversized digital/static spectaculars — quote only, high-end</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Traditional + digital billboards in high-visibility locations.</t>
+          <t>Premier oversized billboard spectaculars at Times Sq, Penn Plaza &amp; Madison Square Garden.</t>
         </is>
       </c>
       <c r="P38" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>silvercastmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Big Outdoor</t>
+          <t>Adams Outdoor Advertising</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>New York (digital spectaculars)</t>
+          <t>New York DMA + mid-size US markets</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -3195,24 +3203,16 @@
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr"/>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G39" s="5" t="inlineStr"/>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr"/>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="inlineStr"/>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>https://bigoutdoor.com/</t>
-        </is>
-      </c>
+      <c r="L39" s="5" t="inlineStr"/>
       <c r="M39" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3220,12 +3220,12 @@
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Digital spectacular — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>NYC digital billboard / spectacular operator.</t>
+          <t>Traditional + digital billboards in high-visibility locations.</t>
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr">
@@ -3242,22 +3242,22 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Billboards America</t>
+          <t>Albert Outdoor Advertising</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
+          <t>Dallas–Fort Worth</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3269,17 +3269,13 @@
       <c r="G40" s="5" t="inlineStr"/>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr"/>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="inlineStr"/>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
-        </is>
-      </c>
+      <c r="L40" s="5" t="inlineStr"/>
       <c r="M40" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3292,12 +3288,12 @@
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>Brokerage with access to prime TX billboard locations.</t>
+          <t>DFW independent operator (named among AdQuick's aggregated DFW operators).</t>
         </is>
       </c>
       <c r="P40" s="5" t="inlineStr">
         <is>
-          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
@@ -3309,22 +3305,22 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Bray Outdoor Ads</t>
+          <t>Avail Media Group</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Houston (independent OOH agency)</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3333,10 +3329,14 @@
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr"/>
-      <c r="G41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://brayoutdoor.com/los-angeles-county/los-angeles-billboards/</t>
+          <t>https://www.availmediagroup.com/capabilities/out-of-home</t>
         </is>
       </c>
       <c r="M41" s="5" t="inlineStr">
@@ -3354,17 +3354,17 @@
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Independent agency — negotiates across vendors</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>LA-county billboard operator/agency.</t>
+          <t>Independent agency negotiating across multiple Houston OOH vendors for placement &amp; pricing.</t>
         </is>
       </c>
       <c r="P41" s="5" t="inlineStr">
         <is>
-          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
+          <t>availmediagroup.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q41" s="5" t="inlineStr">
@@ -3376,7 +3376,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>GreenSigns Chicago</t>
+          <t>Big Outdoor</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -3386,12 +3386,12 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Chicago (all-digital network)</t>
+          <t>New York (digital spectaculars)</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -3402,18 +3402,22 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr"/>
       <c r="J42" s="5" t="inlineStr"/>
       <c r="K42" s="5" t="inlineStr"/>
-      <c r="L42" s="5" t="inlineStr"/>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>https://bigoutdoor.com/</t>
+        </is>
+      </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3421,12 +3425,12 @@
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Digital billboard — quote only</t>
+          <t>Digital spectacular — quote only</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>Fully digital, eco-friendly billboard network.</t>
+          <t>NYC digital billboard / spectacular operator.</t>
         </is>
       </c>
       <c r="P42" s="5" t="inlineStr">
@@ -3443,22 +3447,22 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>GSB Digital</t>
+          <t>Billboards America</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>New York — wildposting / wheatpaste, print &amp; install</t>
+          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston; Dallas; San Antonio</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -3467,14 +3471,10 @@
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr"/>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G43" s="5" t="inlineStr"/>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr"/>
@@ -3482,7 +3482,7 @@
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>https://gsbdigital.com/</t>
+          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
         </is>
       </c>
       <c r="M43" s="5" t="inlineStr">
@@ -3492,17 +3492,17 @@
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Wildposting / production — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O43" s="5" t="inlineStr">
         <is>
-          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
+          <t>Brokerage with access to prime TX billboard locations.</t>
         </is>
       </c>
       <c r="P43" s="5" t="inlineStr">
         <is>
-          <t>gsbdigital.com; WebSearch 2026-07-08</t>
+          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q43" s="5" t="inlineStr">
@@ -3514,7 +3514,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Heritage Outdoor Media</t>
+          <t>Bray Outdoor Ads</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -3524,12 +3524,12 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>New York (Times Square digital)</t>
+          <t>Los Angeles County</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -3538,20 +3538,20 @@
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr"/>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G44" s="5" t="inlineStr"/>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr"/>
       <c r="J44" s="5" t="inlineStr"/>
       <c r="K44" s="5" t="inlineStr"/>
-      <c r="L44" s="5" t="inlineStr"/>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>https://brayoutdoor.com/los-angeles-county/los-angeles-billboards/</t>
+        </is>
+      </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3559,17 +3559,17 @@
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>Times Square digital — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>Times Square LED billboard technology.</t>
+          <t>LA-county billboard operator/agency.</t>
         </is>
       </c>
       <c r="P44" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q44" s="5" t="inlineStr">
@@ -3581,22 +3581,22 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>J&amp;B Signs Inc</t>
+          <t>Dallas Billboards LLC</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Dallas–Fort Worth Metroplex</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3607,18 +3607,22 @@
       <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr"/>
       <c r="J45" s="5" t="inlineStr"/>
       <c r="K45" s="5" t="inlineStr"/>
-      <c r="L45" s="5" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dallasbillboards.com/</t>
+        </is>
+      </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3626,17 +3630,17 @@
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Media buyer / creative agency — quote only</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr">
         <is>
-          <t>Independent OOH media company partnering with local/regional/national advertisers.</t>
+          <t>Full-service OOH media buyer &amp; creative agency securing DFW billboard locations.</t>
         </is>
       </c>
       <c r="P45" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>dallasbillboards.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q45" s="5" t="inlineStr">
@@ -3648,7 +3652,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>MH Outdoor Media</t>
+          <t>GreenSigns Chicago</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -3658,12 +3662,12 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>Chicago (all-digital network)</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3674,12 +3678,12 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr"/>
@@ -3693,12 +3697,12 @@
       </c>
       <c r="N46" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Digital billboard — quote only</t>
         </is>
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>Local Houston billboard operator.</t>
+          <t>Fully digital, eco-friendly billboard network.</t>
         </is>
       </c>
       <c r="P46" s="5" t="inlineStr">
@@ -3715,7 +3719,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Neutron Media</t>
+          <t>GSB Digital</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -3725,7 +3729,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>New York (digital billboards)</t>
+          <t>New York — wildposting / wheatpaste, print &amp; install</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -3752,7 +3756,11 @@
       <c r="I47" s="5" t="inlineStr"/>
       <c r="J47" s="5" t="inlineStr"/>
       <c r="K47" s="5" t="inlineStr"/>
-      <c r="L47" s="5" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>https://gsbdigital.com/</t>
+        </is>
+      </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3760,17 +3768,17 @@
       </c>
       <c r="N47" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Wildposting / production — quote only</t>
         </is>
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
-          <t>Digital billboards in NYC's busiest corridors.</t>
+          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
         </is>
       </c>
       <c r="P47" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>gsbdigital.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q47" s="5" t="inlineStr">
@@ -3782,7 +3790,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>O Media Group</t>
+          <t>Heritage Outdoor Media</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -3792,12 +3800,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York (Times Square digital)</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -3808,12 +3816,12 @@
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr"/>
@@ -3827,12 +3835,12 @@
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Times Square digital — quote only</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
-          <t>LA independent OOH operator (named among Regency's LA competitors).</t>
+          <t>Times Square LED billboard technology.</t>
         </is>
       </c>
       <c r="P48" s="5" t="inlineStr">
@@ -3849,22 +3857,22 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Pearl Media</t>
+          <t>Inspiria Outdoor Advertising</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>New York / Times Square + experiential</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -3875,12 +3883,12 @@
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
@@ -3888,7 +3896,7 @@
       <c r="K49" s="5" t="inlineStr"/>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>https://pearlmedia.com/</t>
+          <t>https://inspiriaoutdoor.com/houston-advertising/</t>
         </is>
       </c>
       <c r="M49" s="5" t="inlineStr">
@@ -3898,17 +3906,17 @@
       </c>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>Times Square / experiential — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr">
         <is>
-          <t>Times Square billboards and experiential activations.</t>
+          <t>Houston billboard advertising across various outdoor formats.</t>
         </is>
       </c>
       <c r="P49" s="5" t="inlineStr">
         <is>
-          <t>pearlmedia.com; WebSearch 2026-07-08</t>
+          <t>inspiriaoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q49" s="5" t="inlineStr">
@@ -3920,22 +3928,22 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Premier Mobile Billboards</t>
+          <t>J&amp;B Signs Inc</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -3946,22 +3954,18 @@
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="inlineStr"/>
       <c r="K50" s="5" t="inlineStr"/>
-      <c r="L50" s="5" t="inlineStr">
-        <is>
-          <t>https://premiermobilebillboards.com/houston/</t>
-        </is>
-      </c>
+      <c r="L50" s="5" t="inlineStr"/>
       <c r="M50" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3969,17 +3973,17 @@
       </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>Digital billboard trucks; Houston + Woodlands, Sugar Land, Katy.</t>
+          <t>Independent OOH media company partnering with local/regional/national advertisers.</t>
         </is>
       </c>
       <c r="P50" s="5" t="inlineStr">
         <is>
-          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q50" s="5" t="inlineStr">
@@ -3991,7 +3995,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Red Rock Outdoor Advertising</t>
+          <t>MH Outdoor Media</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -4001,12 +4005,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>New York (Manhattan)</t>
+          <t>Houston metro</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -4017,12 +4021,12 @@
       <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr"/>
@@ -4041,12 +4045,12 @@
       </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Local Houston billboard operator.</t>
         </is>
       </c>
       <c r="P51" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q51" s="5" t="inlineStr">
@@ -4058,22 +4062,22 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Red Star Outdoor</t>
+          <t>Neutron Media</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York (digital billboards)</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -4084,12 +4088,12 @@
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr"/>
@@ -4108,7 +4112,7 @@
       </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
-          <t>Chicago-market billboard operator (named among major Chicago operators).</t>
+          <t>Digital billboards in NYC's busiest corridors.</t>
         </is>
       </c>
       <c r="P52" s="5" t="inlineStr">
@@ -4125,22 +4129,22 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Rolling Adz Mobile Billboards</t>
+          <t>O Media Group</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>New York City (mobile)</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -4151,22 +4155,18 @@
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr"/>
       <c r="J53" s="5" t="inlineStr"/>
       <c r="K53" s="5" t="inlineStr"/>
-      <c r="L53" s="5" t="inlineStr">
-        <is>
-          <t>https://rollingadz.com/</t>
-        </is>
-      </c>
+      <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4174,17 +4174,17 @@
       </c>
       <c r="N53" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard — day/route rate, quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard fleet across NYC.</t>
+          <t>LA independent OOH operator (named among Regency's LA competitors).</t>
         </is>
       </c>
       <c r="P53" s="5" t="inlineStr">
         <is>
-          <t>rollingadz.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q53" s="5" t="inlineStr">
@@ -4196,17 +4196,17 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Seen Outdoor Media, LLC</t>
+          <t>Pearl Media</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>New York (Brooklyn)</t>
+          <t>New York / Times Square + experiential</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -4222,7 +4222,7 @@
       <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -4233,7 +4233,11 @@
       <c r="I54" s="5" t="inlineStr"/>
       <c r="J54" s="5" t="inlineStr"/>
       <c r="K54" s="5" t="inlineStr"/>
-      <c r="L54" s="5" t="inlineStr"/>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>https://pearlmedia.com/</t>
+        </is>
+      </c>
       <c r="M54" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4241,17 +4245,17 @@
       </c>
       <c r="N54" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Times Square / experiential — quote only</t>
         </is>
       </c>
       <c r="O54" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Times Square billboards and experiential activations.</t>
         </is>
       </c>
       <c r="P54" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>pearlmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q54" s="5" t="inlineStr">
@@ -4263,22 +4267,22 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>TSX Broadway (TSX Entertainment)</t>
+          <t>Premier Mobile Billboards</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Times Square (single landmark asset)</t>
+          <t>Houston; Dallas; San Antonio (mobile)</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston; Dallas; San Antonio</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -4289,18 +4293,22 @@
       <c r="F55" s="5" t="inlineStr"/>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr"/>
       <c r="J55" s="5" t="inlineStr"/>
       <c r="K55" s="5" t="inlineStr"/>
-      <c r="L55" s="5" t="inlineStr"/>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>https://premiermobilebillboards.com/</t>
+        </is>
+      </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4308,17 +4316,17 @@
       </c>
       <c r="N55" s="5" t="inlineStr">
         <is>
-          <t>Premium spectacular — quote only, very high-end</t>
+          <t>Mobile LED truck — quote only</t>
         </is>
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>Flagship 18k-sq-ft curved LED at 47th &amp; Broadway, Times Square.</t>
+          <t>Digital billboard trucks across major TX metros (Houston, Dallas, San Antonio).</t>
         </is>
       </c>
       <c r="P55" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q55" s="5" t="inlineStr">
@@ -4330,22 +4338,22 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>VC Outdoor</t>
+          <t>Ralston Outdoor Advertising</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Chicago (40 neighborhoods)</t>
+          <t>Dallas–Fort Worth</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -4354,14 +4362,10 @@
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr"/>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
+      <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr"/>
@@ -4375,27 +4379,500 @@
       </c>
       <c r="N56" s="5" t="inlineStr">
         <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O56" s="5" t="inlineStr">
+        <is>
+          <t>DFW independent operator (inventory aggregated by AdQuick alongside Lamar/CCO/OUTFRONT).</t>
+        </is>
+      </c>
+      <c r="P56" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Red Rock Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>New York (Manhattan)</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr"/>
+      <c r="J57" s="5" t="inlineStr"/>
+      <c r="K57" s="5" t="inlineStr"/>
+      <c r="L57" s="5" t="inlineStr"/>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N57" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O57" s="5" t="inlineStr">
+        <is>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+        </is>
+      </c>
+      <c r="P57" s="5" t="inlineStr">
+        <is>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Red Star Outdoor</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr"/>
+      <c r="J58" s="5" t="inlineStr"/>
+      <c r="K58" s="5" t="inlineStr"/>
+      <c r="L58" s="5" t="inlineStr"/>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N58" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O58" s="5" t="inlineStr">
+        <is>
+          <t>Chicago-market billboard operator (named among major Chicago operators).</t>
+        </is>
+      </c>
+      <c r="P58" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q58" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Rolling Adz Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>New York City (mobile)</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr"/>
+      <c r="J59" s="5" t="inlineStr"/>
+      <c r="K59" s="5" t="inlineStr"/>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>https://rollingadz.com/</t>
+        </is>
+      </c>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N59" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard — day/route rate, quote only</t>
+        </is>
+      </c>
+      <c r="O59" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard fleet across NYC.</t>
+        </is>
+      </c>
+      <c r="P59" s="5" t="inlineStr">
+        <is>
+          <t>rollingadz.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Seen Outdoor Media, LLC</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>New York (Brooklyn)</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr"/>
+      <c r="J60" s="5" t="inlineStr"/>
+      <c r="K60" s="5" t="inlineStr"/>
+      <c r="L60" s="5" t="inlineStr"/>
+      <c r="M60" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N60" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O60" s="5" t="inlineStr">
+        <is>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+        </is>
+      </c>
+      <c r="P60" s="5" t="inlineStr">
+        <is>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>True Impact Media</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Broker / agency / marketplace</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio (+ national mobile)</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr"/>
+      <c r="J61" s="5" t="inlineStr"/>
+      <c r="K61" s="5" t="inlineStr"/>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>https://trueimpactmedia.com/billboard-advertising-in-san-antonio/</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N61" s="5" t="inlineStr">
+        <is>
+          <t>Billboards + mobile — quote only</t>
+        </is>
+      </c>
+      <c r="O61" s="5" t="inlineStr">
+        <is>
+          <t>Comprehensive San Antonio OOH incl. static, digital and mobile billboards.</t>
+        </is>
+      </c>
+      <c r="P61" s="5" t="inlineStr">
+        <is>
+          <t>trueimpactmedia.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>TSX Broadway (TSX Entertainment)</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Times Square (single landmark asset)</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr"/>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
+      <c r="M62" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N62" s="5" t="inlineStr">
+        <is>
+          <t>Premium spectacular — quote only, very high-end</t>
+        </is>
+      </c>
+      <c r="O62" s="5" t="inlineStr">
+        <is>
+          <t>Flagship 18k-sq-ft curved LED at 47th &amp; Broadway, Times Square.</t>
+        </is>
+      </c>
+      <c r="P62" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>VC Outdoor</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Chicago (40 neighborhoods)</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr"/>
+      <c r="J63" s="5" t="inlineStr"/>
+      <c r="K63" s="5" t="inlineStr"/>
+      <c r="L63" s="5" t="inlineStr"/>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N63" s="5" t="inlineStr">
+        <is>
           <t>Wildposting / wallscape / bus wrap — quote only</t>
         </is>
       </c>
-      <c r="O56" s="5" t="inlineStr">
+      <c r="O63" s="5" t="inlineStr">
         <is>
           <t>Hotspots, wild postings, wallscapes, bus wraps &amp; street furniture across 40 Chicago neighborhoods.</t>
         </is>
       </c>
-      <c r="P56" s="5" t="inlineStr">
+      <c r="P63" s="5" t="inlineStr">
         <is>
           <t>WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q56" s="5" t="inlineStr">
+      <c r="Q63" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q56"/>
+  <autoFilter ref="A4:Q63"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -5172,7 +5649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5204,7 +5681,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>11 companies serving Dallas · prices quote-only</t>
+          <t>16 companies serving Dallas · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -5858,7 +6335,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>BM Outdoor Media</t>
+          <t>Arrington Outdoor Advertising</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -5868,12 +6345,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>44 Texas cities + Phoenix</t>
+          <t>Dallas–Fort Worth Metroplex</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio; Phoenix</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -5882,10 +6359,14 @@
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
@@ -5893,7 +6374,7 @@
       <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://bmoutdoor.com/</t>
+          <t>https://www.arringtonoutdoor.com/</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -5908,12 +6389,12 @@
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
+          <t>Largest independent billboard company in the DFW area; bulletins &amp; digital.</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>bmoutdoor.com; WebSearch 2026-07-08</t>
+          <t>arringtonoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q13" s="5" t="inlineStr">
@@ -5925,22 +6406,22 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Lux Media</t>
+          <t>BM Outdoor Media</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Dallas; Houston; Austin; San Antonio</t>
+          <t>44 Texas cities + Phoenix</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Houston; San Antonio; Dallas</t>
+          <t>Houston; Dallas; San Antonio; Phoenix</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -5960,7 +6441,7 @@
       <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>https://www.luxmediaads.com/</t>
+          <t>https://bmoutdoor.com/</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
@@ -5970,17 +6451,17 @@
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — day/route rate, quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED billboard truck advertising across major TX metros.</t>
+          <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>luxmediaads.com; WebSearch 2026-07-08</t>
+          <t>bmoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
@@ -5992,22 +6473,22 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Billboards America</t>
+          <t>Lux Media</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
+          <t>Dallas; Houston; Austin; San Antonio</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio</t>
+          <t>Houston; San Antonio; Dallas</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -6027,37 +6508,372 @@
       <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="5" t="inlineStr">
         <is>
+          <t>https://www.luxmediaads.com/</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — day/route rate, quote only</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED billboard truck advertising across major TX metros.</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>luxmediaads.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Albert Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Dallas–Fort Worth</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>DFW independent operator (named among AdQuick's aggregated DFW operators).</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Billboards America</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Broker / agency / marketplace</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
           <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
-        <is>
-          <t>Quote only — request from company</t>
-        </is>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
-      <c r="O15" s="5" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>Brokerage with access to prime TX billboard locations.</t>
         </is>
       </c>
-      <c r="P15" s="5" t="inlineStr">
+      <c r="P17" s="5" t="inlineStr">
         <is>
           <t>billboardsamerica.com; WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q15" s="5" t="inlineStr">
+      <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Billboards LLC</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Broker / agency / marketplace</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Dallas–Fort Worth Metroplex</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dallasbillboards.com/</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Media buyer / creative agency — quote only</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Full-service OOH media buyer &amp; creative agency securing DFW billboard locations.</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>dallasbillboards.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Premier Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio (mobile)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>https://premiermobilebillboards.com/</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — quote only</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboard trucks across major TX metros (Houston, Dallas, San Antonio).</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Ralston Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Dallas–Fort Worth</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>DFW independent operator (inventory aggregated by AdQuick alongside Lamar/CCO/OUTFRONT).</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q15"/>
+  <autoFilter ref="A4:Q20"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -7085,7 +7901,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Generated by fbscraper v1.0 · 52 companies · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville.</t>
+          <t>Generated by fbscraper v1.0 · 59 companies · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville.</t>
         </is>
       </c>
     </row>
@@ -12822,7 +13638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12854,7 +13670,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>14 companies serving Houston · prices quote-only</t>
+          <t>16 companies serving Houston · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -13713,7 +14529,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Billboards America</t>
+          <t>Avail Media Group</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -13723,12 +14539,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
+          <t>Houston (independent OOH agency)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -13737,10 +14553,14 @@
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
-      <c r="G16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr"/>
@@ -13748,7 +14568,7 @@
       <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
+          <t>https://www.availmediagroup.com/capabilities/out-of-home</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
@@ -13758,17 +14578,17 @@
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Independent agency — negotiates across vendors</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>Brokerage with access to prime TX billboard locations.</t>
+          <t>Independent agency negotiating across multiple Houston OOH vendors for placement &amp; pricing.</t>
         </is>
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
+          <t>availmediagroup.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
@@ -13780,22 +14600,22 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>MH Outdoor Media</t>
+          <t>Billboards America</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Houston; Dallas; San Antonio</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -13804,20 +14624,20 @@
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
+      <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
+        </is>
+      </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -13830,12 +14650,12 @@
       </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
-          <t>Local Houston billboard operator.</t>
+          <t>Brokerage with access to prime TX billboard locations.</t>
         </is>
       </c>
       <c r="P17" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q17" s="5" t="inlineStr">
@@ -13847,17 +14667,17 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Premier Mobile Billboards</t>
+          <t>Inspiria Outdoor Advertising</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -13886,7 +14706,7 @@
       <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>https://premiermobilebillboards.com/houston/</t>
+          <t>https://inspiriaoutdoor.com/houston-advertising/</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
@@ -13896,27 +14716,165 @@
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Houston billboard advertising across various outdoor formats.</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>inspiriaoutdoor.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>MH Outdoor Media</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Houston metro</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr"/>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Local Houston billboard operator.</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Premier Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio (mobile)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>https://premiermobilebillboards.com/</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
           <t>Mobile LED truck — quote only</t>
         </is>
       </c>
-      <c r="O18" s="5" t="inlineStr">
-        <is>
-          <t>Digital billboard trucks; Houston + Woodlands, Sugar Land, Katy.</t>
-        </is>
-      </c>
-      <c r="P18" s="5" t="inlineStr">
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboard trucks across major TX metros (Houston, Dallas, San Antonio).</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
         <is>
           <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q18" s="5" t="inlineStr">
+      <c r="Q20" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q18"/>
+  <autoFilter ref="A4:Q20"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -15601,7 +16559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -15633,7 +16591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>12 companies serving San Antonio · prices quote-only</t>
+          <t>14 companies serving San Antonio · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -16556,8 +17514,146 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Premier Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio (mobile)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>https://premiermobilebillboards.com/</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — quote only</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboard trucks across major TX metros (Houston, Dallas, San Antonio).</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>True Impact Media</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Broker / agency / marketplace</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio (+ national mobile)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>https://trueimpactmedia.com/billboard-advertising-in-san-antonio/</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Billboards + mobile — quote only</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Comprehensive San Antonio OOH incl. static, digital and mobile billboards.</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>trueimpactmedia.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q16"/>
+  <autoFilter ref="A4:Q18"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>

</xml_diff>

<commit_message>
Deep-dive final 4 markets: all 10 cities now have local operators (total 64)
- Philadelphia (13): add Catalyst Outdoor (w/ 2024 distress note), Keystone
  Outdoor; broaden Big Outdoor to Philadelphia.
- Jacksonville (12): add Daily Billboards, American Mobile Ads, Fisher Design.
- Phoenix (11) / San Diego (10): broaden American Outdoor (SD+Phoenix) and
  Bray Outdoor (LA+SD) coverage.
- Every one of the 10 cities now lists local operators, not just nationals.
- README updated with full per-city depth.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169X7FqU7js4G1ZKY5WjVsV
</commit_message>
<xml_diff>
--- a/florida-billboard-scraper/data/us_top_cities_billboard_companies.xlsx
+++ b/florida-billboard-scraper/data/us_top_cities_billboard_companies.xlsx
@@ -23,17 +23,17 @@
     <sheet name="About" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Companies'!$A$4:$Q$63</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New York'!$A$4:$Q$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Companies'!$A$4:$Q$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New York'!$A$4:$Q$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Los Angeles'!$A$4:$Q$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Chicago'!$A$4:$Q$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Houston'!$A$4:$Q$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Phoenix'!$A$4:$Q$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Philadelphia'!$A$4:$Q$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Phoenix'!$A$4:$Q$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Philadelphia'!$A$4:$Q$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'San Antonio'!$A$4:$Q$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'San Diego'!$A$4:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'San Diego'!$A$4:$Q$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Dallas'!$A$4:$Q$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Jacksonville'!$A$4:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Jacksonville'!$A$4:$Q$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q63"/>
+  <dimension ref="A1:Q68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -703,7 +703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>59 companies · national operators first · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville</t>
+          <t>64 companies · national operators first · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville</t>
         </is>
       </c>
     </row>
@@ -2215,12 +2215,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Diego; Phoenix</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Diego; Phoenix</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>Digital &amp; static billboards on high-traffic San Diego routes.</t>
+          <t>Digital &amp; static billboards on high-traffic routes; regional operator in San Diego and Phoenix.</t>
         </is>
       </c>
       <c r="P25" s="5" t="inlineStr">
@@ -3305,22 +3305,22 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Avail Media Group</t>
+          <t>American Mobile Ads</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Houston (independent OOH agency)</t>
+          <t>Jacksonville (mobile)</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3329,14 +3329,10 @@
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr"/>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
+      <c r="G41" s="5" t="inlineStr"/>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr"/>
@@ -3344,7 +3340,7 @@
       <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://www.availmediagroup.com/capabilities/out-of-home</t>
+          <t>https://americanmobileads.com/markets/jacksonville</t>
         </is>
       </c>
       <c r="M41" s="5" t="inlineStr">
@@ -3354,17 +3350,17 @@
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Independent agency — negotiates across vendors</t>
+          <t>Mobile LED truck — day/route rate, quote only</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>Independent agency negotiating across multiple Houston OOH vendors for placement &amp; pricing.</t>
+          <t>Backlit + digital LED/video mobile billboard trucks in Jacksonville.</t>
         </is>
       </c>
       <c r="P41" s="5" t="inlineStr">
         <is>
-          <t>availmediagroup.com; WebSearch 2026-07-08</t>
+          <t>americanmobileads.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q41" s="5" t="inlineStr">
@@ -3376,22 +3372,22 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Big Outdoor</t>
+          <t>Avail Media Group</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>New York (digital spectaculars)</t>
+          <t>Houston (independent OOH agency)</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -3402,12 +3398,12 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr"/>
@@ -3415,7 +3411,7 @@
       <c r="K42" s="5" t="inlineStr"/>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>https://bigoutdoor.com/</t>
+          <t>https://www.availmediagroup.com/capabilities/out-of-home</t>
         </is>
       </c>
       <c r="M42" s="5" t="inlineStr">
@@ -3425,17 +3421,17 @@
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Digital spectacular — quote only</t>
+          <t>Independent agency — negotiates across vendors</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>NYC digital billboard / spectacular operator.</t>
+          <t>Independent agency negotiating across multiple Houston OOH vendors for placement &amp; pricing.</t>
         </is>
       </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>availmediagroup.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q42" s="5" t="inlineStr">
@@ -3447,22 +3443,22 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Billboards America</t>
+          <t>Big Outdoor</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
+          <t>New York; Philadelphia (digital spectaculars)</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio</t>
+          <t>New York; Philadelphia</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -3471,10 +3467,14 @@
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr"/>
-      <c r="G43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr"/>
@@ -3482,7 +3482,7 @@
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
+          <t>https://bigoutdoor.com/</t>
         </is>
       </c>
       <c r="M43" s="5" t="inlineStr">
@@ -3492,17 +3492,17 @@
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Digital spectacular — quote only</t>
         </is>
       </c>
       <c r="O43" s="5" t="inlineStr">
         <is>
-          <t>Brokerage with access to prime TX billboard locations.</t>
+          <t>Digital billboard / spectacular operator (NYC + Philadelphia).</t>
         </is>
       </c>
       <c r="P43" s="5" t="inlineStr">
         <is>
-          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q43" s="5" t="inlineStr">
@@ -3514,22 +3514,22 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Bray Outdoor Ads</t>
+          <t>Billboards America</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Texas (Dallas, Houston, Austin, San Antonio, Fort Worth)</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston; Dallas; San Antonio</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -3549,7 +3549,7 @@
       <c r="K44" s="5" t="inlineStr"/>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>https://brayoutdoor.com/los-angeles-county/los-angeles-billboards/</t>
+          <t>https://www.billboardsamerica.com/billboard-advertising-locations/texas</t>
         </is>
       </c>
       <c r="M44" s="5" t="inlineStr">
@@ -3564,12 +3564,12 @@
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>LA-county billboard operator/agency.</t>
+          <t>Brokerage with access to prime TX billboard locations.</t>
         </is>
       </c>
       <c r="P44" s="5" t="inlineStr">
         <is>
-          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
+          <t>billboardsamerica.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q44" s="5" t="inlineStr">
@@ -3581,22 +3581,22 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Dallas Billboards LLC</t>
+          <t>Bray Outdoor Ads</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Dallas–Fort Worth Metroplex</t>
+          <t>Los Angeles &amp; San Diego counties (SoCal)</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Los Angeles; San Diego</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3605,14 +3605,10 @@
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr"/>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Dallas</t>
-        </is>
-      </c>
+      <c r="G45" s="5" t="inlineStr"/>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr"/>
@@ -3620,7 +3616,7 @@
       <c r="K45" s="5" t="inlineStr"/>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>https://www.dallasbillboards.com/</t>
+          <t>https://brayoutdoor.com/</t>
         </is>
       </c>
       <c r="M45" s="5" t="inlineStr">
@@ -3630,17 +3626,17 @@
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Media buyer / creative agency — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr">
         <is>
-          <t>Full-service OOH media buyer &amp; creative agency securing DFW billboard locations.</t>
+          <t>SoCal billboard operator/media buyer across LA and San Diego counties.</t>
         </is>
       </c>
       <c r="P45" s="5" t="inlineStr">
         <is>
-          <t>dallasbillboards.com; WebSearch 2026-07-08</t>
+          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q45" s="5" t="inlineStr">
@@ -3652,22 +3648,22 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>GreenSigns Chicago</t>
+          <t>Catalyst Outdoor Advertising</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Chicago (all-digital network)</t>
+          <t>Philadelphia suburbs + New York</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Philadelphia; New York</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3676,20 +3672,20 @@
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr"/>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
+      <c r="G46" s="5" t="inlineStr"/>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr"/>
       <c r="J46" s="5" t="inlineStr"/>
       <c r="K46" s="5" t="inlineStr"/>
-      <c r="L46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/catalyst-outdoor-advertising</t>
+        </is>
+      </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3697,17 +3693,17 @@
       </c>
       <c r="N46" s="5" t="inlineStr">
         <is>
-          <t>Digital billboard — quote only</t>
+          <t>Digital billboards — quote only</t>
         </is>
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>Fully digital, eco-friendly billboard network.</t>
+          <t>Founded 2009 (Thaddeus Bartkowski); ~14 digital faces, known for 'living wall' displays. NOTE: financial distress in 2024; assets reportedly being sold to Lamar &amp; Clear Channel — verify current ownership before contacting.</t>
         </is>
       </c>
       <c r="P46" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>Billboard Insider; Philadelphia Inquirer; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q46" s="5" t="inlineStr">
@@ -3719,7 +3715,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>GSB Digital</t>
+          <t>Daily Billboards</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -3729,12 +3725,12 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>New York — wildposting / wheatpaste, print &amp; install</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -3745,22 +3741,18 @@
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr"/>
       <c r="J47" s="5" t="inlineStr"/>
       <c r="K47" s="5" t="inlineStr"/>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>https://gsbdigital.com/</t>
-        </is>
-      </c>
+      <c r="L47" s="5" t="inlineStr"/>
       <c r="M47" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3768,17 +3760,17 @@
       </c>
       <c r="N47" s="5" t="inlineStr">
         <is>
-          <t>Wildposting / production — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
-          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
+          <t>Independent operator with ~49 billboard locations in and around Jacksonville.</t>
         </is>
       </c>
       <c r="P47" s="5" t="inlineStr">
         <is>
-          <t>gsbdigital.com; WebSearch 2026-07-08</t>
+          <t>Alignable; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q47" s="5" t="inlineStr">
@@ -3790,22 +3782,22 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Heritage Outdoor Media</t>
+          <t>Dallas Billboards LLC</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>New York (Times Square digital)</t>
+          <t>Dallas–Fort Worth Metroplex</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -3816,18 +3808,22 @@
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr"/>
       <c r="J48" s="5" t="inlineStr"/>
       <c r="K48" s="5" t="inlineStr"/>
-      <c r="L48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dallasbillboards.com/</t>
+        </is>
+      </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -3835,17 +3831,17 @@
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>Times Square digital — quote only</t>
+          <t>Media buyer / creative agency — quote only</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
-          <t>Times Square LED billboard technology.</t>
+          <t>Full-service OOH media buyer &amp; creative agency securing DFW billboard locations.</t>
         </is>
       </c>
       <c r="P48" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>dallasbillboards.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q48" s="5" t="inlineStr">
@@ -3857,22 +3853,22 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Inspiria Outdoor Advertising</t>
+          <t>Fisher Design &amp; Advertising</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Jacksonville (agency)</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -3883,12 +3879,12 @@
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
@@ -3896,7 +3892,7 @@
       <c r="K49" s="5" t="inlineStr"/>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>https://inspiriaoutdoor.com/houston-advertising/</t>
+          <t>https://www.fisherdesignandadvertising.com/services/outdoor-advertising-jacksonville/</t>
         </is>
       </c>
       <c r="M49" s="5" t="inlineStr">
@@ -3906,17 +3902,17 @@
       </c>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Agency — books across outdoor vendors, quote only</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr">
         <is>
-          <t>Houston billboard advertising across various outdoor formats.</t>
+          <t>Agency partnering with outdoor companies for Jacksonville OOH campaigns.</t>
         </is>
       </c>
       <c r="P49" s="5" t="inlineStr">
         <is>
-          <t>inspiriaoutdoor.com; WebSearch 2026-07-08</t>
+          <t>fisherdesignandadvertising.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q49" s="5" t="inlineStr">
@@ -3928,7 +3924,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>J&amp;B Signs Inc</t>
+          <t>GreenSigns Chicago</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -3938,7 +3934,7 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chicago (all-digital network)</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -3973,12 +3969,12 @@
       </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Digital billboard — quote only</t>
         </is>
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>Independent OOH media company partnering with local/regional/national advertisers.</t>
+          <t>Fully digital, eco-friendly billboard network.</t>
         </is>
       </c>
       <c r="P50" s="5" t="inlineStr">
@@ -3995,7 +3991,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>MH Outdoor Media</t>
+          <t>GSB Digital</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -4005,12 +4001,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Houston metro</t>
+          <t>New York — wildposting / wheatpaste, print &amp; install</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -4021,18 +4017,22 @@
       <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr"/>
       <c r="J51" s="5" t="inlineStr"/>
       <c r="K51" s="5" t="inlineStr"/>
-      <c r="L51" s="5" t="inlineStr"/>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>https://gsbdigital.com/</t>
+        </is>
+      </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4040,17 +4040,17 @@
       </c>
       <c r="N51" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Wildposting / production — quote only</t>
         </is>
       </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
-          <t>Local Houston billboard operator.</t>
+          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
         </is>
       </c>
       <c r="P51" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>gsbdigital.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q51" s="5" t="inlineStr">
@@ -4062,7 +4062,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Neutron Media</t>
+          <t>Heritage Outdoor Media</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>New York (digital billboards)</t>
+          <t>New York (Times Square digital)</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="N52" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Times Square digital — quote only</t>
         </is>
       </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
-          <t>Digital billboards in NYC's busiest corridors.</t>
+          <t>Times Square LED billboard technology.</t>
         </is>
       </c>
       <c r="P52" s="5" t="inlineStr">
@@ -4129,7 +4129,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>O Media Group</t>
+          <t>Inspiria Outdoor Advertising</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -4139,12 +4139,12 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -4155,18 +4155,22 @@
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr"/>
       <c r="J53" s="5" t="inlineStr"/>
       <c r="K53" s="5" t="inlineStr"/>
-      <c r="L53" s="5" t="inlineStr"/>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>https://inspiriaoutdoor.com/houston-advertising/</t>
+        </is>
+      </c>
       <c r="M53" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4179,12 +4183,12 @@
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
-          <t>LA independent OOH operator (named among Regency's LA competitors).</t>
+          <t>Houston billboard advertising across various outdoor formats.</t>
         </is>
       </c>
       <c r="P53" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>inspiriaoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q53" s="5" t="inlineStr">
@@ -4196,22 +4200,22 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Pearl Media</t>
+          <t>J&amp;B Signs Inc</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>New York / Times Square + experiential</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -4222,22 +4226,18 @@
       <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr"/>
       <c r="J54" s="5" t="inlineStr"/>
       <c r="K54" s="5" t="inlineStr"/>
-      <c r="L54" s="5" t="inlineStr">
-        <is>
-          <t>https://pearlmedia.com/</t>
-        </is>
-      </c>
+      <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4245,17 +4245,17 @@
       </c>
       <c r="N54" s="5" t="inlineStr">
         <is>
-          <t>Times Square / experiential — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O54" s="5" t="inlineStr">
         <is>
-          <t>Times Square billboards and experiential activations.</t>
+          <t>Independent OOH media company partnering with local/regional/national advertisers.</t>
         </is>
       </c>
       <c r="P54" s="5" t="inlineStr">
         <is>
-          <t>pearlmedia.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q54" s="5" t="inlineStr">
@@ -4267,22 +4267,22 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Premier Mobile Billboards</t>
+          <t>Keystone Outdoor Advertising</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio (mobile)</t>
+          <t>Philadelphia / Pennsylvania</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -4291,14 +4291,10 @@
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr"/>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
+      <c r="G55" s="5" t="inlineStr"/>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr"/>
@@ -4306,7 +4302,7 @@
       <c r="K55" s="5" t="inlineStr"/>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>https://premiermobilebillboards.com/</t>
+          <t>https://www.keystoneoutdoor.com/</t>
         </is>
       </c>
       <c r="M55" s="5" t="inlineStr">
@@ -4316,17 +4312,17 @@
       </c>
       <c r="N55" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>Digital billboard trucks across major TX metros (Houston, Dallas, San Antonio).</t>
+          <t>Regional PA billboard operator serving the Philadelphia market.</t>
         </is>
       </c>
       <c r="P55" s="5" t="inlineStr">
         <is>
-          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q55" s="5" t="inlineStr">
@@ -4338,22 +4334,22 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Ralston Outdoor Advertising</t>
+          <t>MH Outdoor Media</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Dallas–Fort Worth</t>
+          <t>Houston metro</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -4362,7 +4358,11 @@
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr"/>
-      <c r="G56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
           <t>TX</t>
@@ -4384,7 +4384,7 @@
       </c>
       <c r="O56" s="5" t="inlineStr">
         <is>
-          <t>DFW independent operator (inventory aggregated by AdQuick alongside Lamar/CCO/OUTFRONT).</t>
+          <t>Local Houston billboard operator.</t>
         </is>
       </c>
       <c r="P56" s="5" t="inlineStr">
@@ -4401,7 +4401,7 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Red Rock Outdoor Advertising</t>
+          <t>Neutron Media</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>New York (Manhattan)</t>
+          <t>New York (digital billboards)</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -4451,12 +4451,12 @@
       </c>
       <c r="O57" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Digital billboards in NYC's busiest corridors.</t>
         </is>
       </c>
       <c r="P57" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q57" s="5" t="inlineStr">
@@ -4468,22 +4468,22 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Red Star Outdoor</t>
+          <t>O Media Group</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -4494,12 +4494,12 @@
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr"/>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="O58" s="5" t="inlineStr">
         <is>
-          <t>Chicago-market billboard operator (named among major Chicago operators).</t>
+          <t>LA independent OOH operator (named among Regency's LA competitors).</t>
         </is>
       </c>
       <c r="P58" s="5" t="inlineStr">
@@ -4535,17 +4535,17 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Rolling Adz Mobile Billboards</t>
+          <t>Pearl Media</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>New York City (mobile)</t>
+          <t>New York / Times Square + experiential</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -4574,7 +4574,7 @@
       <c r="K59" s="5" t="inlineStr"/>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>https://rollingadz.com/</t>
+          <t>https://pearlmedia.com/</t>
         </is>
       </c>
       <c r="M59" s="5" t="inlineStr">
@@ -4584,17 +4584,17 @@
       </c>
       <c r="N59" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard — day/route rate, quote only</t>
+          <t>Times Square / experiential — quote only</t>
         </is>
       </c>
       <c r="O59" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard fleet across NYC.</t>
+          <t>Times Square billboards and experiential activations.</t>
         </is>
       </c>
       <c r="P59" s="5" t="inlineStr">
         <is>
-          <t>rollingadz.com; WebSearch 2026-07-08</t>
+          <t>pearlmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q59" s="5" t="inlineStr">
@@ -4606,22 +4606,22 @@
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Seen Outdoor Media, LLC</t>
+          <t>Premier Mobile Billboards</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>New York (Brooklyn)</t>
+          <t>Houston; Dallas; San Antonio (mobile)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston; Dallas; San Antonio</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -4632,18 +4632,22 @@
       <c r="F60" s="5" t="inlineStr"/>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr"/>
       <c r="J60" s="5" t="inlineStr"/>
       <c r="K60" s="5" t="inlineStr"/>
-      <c r="L60" s="5" t="inlineStr"/>
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>https://premiermobilebillboards.com/</t>
+        </is>
+      </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4651,17 +4655,17 @@
       </c>
       <c r="N60" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Mobile LED truck — quote only</t>
         </is>
       </c>
       <c r="O60" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Digital billboard trucks across major TX metros (Houston, Dallas, San Antonio).</t>
         </is>
       </c>
       <c r="P60" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>premiermobilebillboards.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q60" s="5" t="inlineStr">
@@ -4673,22 +4677,22 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>True Impact Media</t>
+          <t>Ralston Outdoor Advertising</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>San Antonio (+ national mobile)</t>
+          <t>Dallas–Fort Worth</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -4700,17 +4704,13 @@
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr"/>
       <c r="J61" s="5" t="inlineStr"/>
       <c r="K61" s="5" t="inlineStr"/>
-      <c r="L61" s="5" t="inlineStr">
-        <is>
-          <t>https://trueimpactmedia.com/billboard-advertising-in-san-antonio/</t>
-        </is>
-      </c>
+      <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -4718,17 +4718,17 @@
       </c>
       <c r="N61" s="5" t="inlineStr">
         <is>
-          <t>Billboards + mobile — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O61" s="5" t="inlineStr">
         <is>
-          <t>Comprehensive San Antonio OOH incl. static, digital and mobile billboards.</t>
+          <t>DFW independent operator (inventory aggregated by AdQuick alongside Lamar/CCO/OUTFRONT).</t>
         </is>
       </c>
       <c r="P61" s="5" t="inlineStr">
         <is>
-          <t>trueimpactmedia.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q61" s="5" t="inlineStr">
@@ -4740,7 +4740,7 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>TSX Broadway (TSX Entertainment)</t>
+          <t>Red Rock Outdoor Advertising</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Times Square (single landmark asset)</t>
+          <t>New York (Manhattan)</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -4785,17 +4785,17 @@
       </c>
       <c r="N62" s="5" t="inlineStr">
         <is>
-          <t>Premium spectacular — quote only, very high-end</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O62" s="5" t="inlineStr">
         <is>
-          <t>Flagship 18k-sq-ft curved LED at 47th &amp; Broadway, Times Square.</t>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
         </is>
       </c>
       <c r="P62" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q62" s="5" t="inlineStr">
@@ -4807,17 +4807,17 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>VC Outdoor</t>
+          <t>Red Star Outdoor</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Chicago (40 neighborhoods)</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -4852,27 +4852,366 @@
       </c>
       <c r="N63" s="5" t="inlineStr">
         <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O63" s="5" t="inlineStr">
+        <is>
+          <t>Chicago-market billboard operator (named among major Chicago operators).</t>
+        </is>
+      </c>
+      <c r="P63" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q63" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Rolling Adz Mobile Billboards</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>New York City (mobile)</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr"/>
+      <c r="J64" s="5" t="inlineStr"/>
+      <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>https://rollingadz.com/</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N64" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard — day/route rate, quote only</t>
+        </is>
+      </c>
+      <c r="O64" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard fleet across NYC.</t>
+        </is>
+      </c>
+      <c r="P64" s="5" t="inlineStr">
+        <is>
+          <t>rollingadz.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Seen Outdoor Media, LLC</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>New York (Brooklyn)</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr"/>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr"/>
+      <c r="J65" s="5" t="inlineStr"/>
+      <c r="K65" s="5" t="inlineStr"/>
+      <c r="L65" s="5" t="inlineStr"/>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N65" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O65" s="5" t="inlineStr">
+        <is>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+        </is>
+      </c>
+      <c r="P65" s="5" t="inlineStr">
+        <is>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>True Impact Media</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Broker / agency / marketplace</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio (+ national mobile)</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="5" t="inlineStr"/>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr"/>
+      <c r="J66" s="5" t="inlineStr"/>
+      <c r="K66" s="5" t="inlineStr"/>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>https://trueimpactmedia.com/billboard-advertising-in-san-antonio/</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N66" s="5" t="inlineStr">
+        <is>
+          <t>Billboards + mobile — quote only</t>
+        </is>
+      </c>
+      <c r="O66" s="5" t="inlineStr">
+        <is>
+          <t>Comprehensive San Antonio OOH incl. static, digital and mobile billboards.</t>
+        </is>
+      </c>
+      <c r="P66" s="5" t="inlineStr">
+        <is>
+          <t>trueimpactmedia.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>TSX Broadway (TSX Entertainment)</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Times Square (single landmark asset)</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr"/>
+      <c r="J67" s="5" t="inlineStr"/>
+      <c r="K67" s="5" t="inlineStr"/>
+      <c r="L67" s="5" t="inlineStr"/>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N67" s="5" t="inlineStr">
+        <is>
+          <t>Premium spectacular — quote only, very high-end</t>
+        </is>
+      </c>
+      <c r="O67" s="5" t="inlineStr">
+        <is>
+          <t>Flagship 18k-sq-ft curved LED at 47th &amp; Broadway, Times Square.</t>
+        </is>
+      </c>
+      <c r="P67" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>VC Outdoor</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Chicago (40 neighborhoods)</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr"/>
+      <c r="J68" s="5" t="inlineStr"/>
+      <c r="K68" s="5" t="inlineStr"/>
+      <c r="L68" s="5" t="inlineStr"/>
+      <c r="M68" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N68" s="5" t="inlineStr">
+        <is>
           <t>Wildposting / wallscape / bus wrap — quote only</t>
         </is>
       </c>
-      <c r="O63" s="5" t="inlineStr">
+      <c r="O68" s="5" t="inlineStr">
         <is>
           <t>Hotspots, wild postings, wallscapes, bus wraps &amp; street furniture across 40 Chicago neighborhoods.</t>
         </is>
       </c>
-      <c r="P63" s="5" t="inlineStr">
+      <c r="P68" s="5" t="inlineStr">
         <is>
           <t>WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q63" s="5" t="inlineStr">
+      <c r="Q68" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q63"/>
+  <autoFilter ref="A4:Q68"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -4887,7 +5226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4919,7 +5258,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>9 companies serving San Diego · prices quote-only</t>
+          <t>10 companies serving San Diego · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -5579,12 +5918,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Diego; Phoenix</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Diego; Phoenix</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -5619,7 +5958,7 @@
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>Digital &amp; static billboards on high-traffic San Diego routes.</t>
+          <t>Digital &amp; static billboards on high-traffic routes; regional operator in San Diego and Phoenix.</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
@@ -5633,8 +5972,75 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Bray Outdoor Ads</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles &amp; San Diego counties (SoCal)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles; San Diego</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>https://brayoutdoor.com/</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>SoCal billboard operator/media buyer across LA and San Diego counties.</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>brayoutdoor.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q13"/>
+  <autoFilter ref="A4:Q14"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -6888,7 +7294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -6920,7 +7326,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>9 companies serving Jacksonville · prices quote-only</t>
+          <t>12 companies serving Jacksonville · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -7634,8 +8040,213 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>American Mobile Ads</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville (mobile)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>https://americanmobileads.com/markets/jacksonville</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — day/route rate, quote only</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Backlit + digital LED/video mobile billboard trucks in Jacksonville.</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>americanmobileads.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Daily Billboards</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr"/>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Independent operator with ~49 billboard locations in and around Jacksonville.</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Alignable; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Fisher Design &amp; Advertising</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Broker / agency / marketplace</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville (agency)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fisherdesignandadvertising.com/services/outdoor-advertising-jacksonville/</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Agency — books across outdoor vendors, quote only</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Agency partnering with outdoor companies for Jacksonville OOH campaigns.</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>fisherdesignandadvertising.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q13"/>
+  <autoFilter ref="A4:Q16"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -7901,7 +8512,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Generated by fbscraper v1.0 · 59 companies · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville.</t>
+          <t>Generated by fbscraper v1.0 · 64 companies · cities: New York, Los Angeles, Chicago, Houston, Phoenix, Philadelphia, San Antonio, San Diego, Dallas, Jacksonville.</t>
         </is>
       </c>
     </row>
@@ -8426,7 +9037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8458,7 +9069,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>29 companies serving New York · prices quote-only</t>
+          <t>30 companies serving New York · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -9950,12 +10561,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>New York (digital spectaculars)</t>
+          <t>New York; Philadelphia (digital spectaculars)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>New York; Philadelphia</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -9994,7 +10605,7 @@
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t>NYC digital billboard / spectacular operator.</t>
+          <t>Digital billboard / spectacular operator (NYC + Philadelphia).</t>
         </is>
       </c>
       <c r="P25" s="5" t="inlineStr">
@@ -10011,22 +10622,22 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>GSB Digital</t>
+          <t>Catalyst Outdoor Advertising</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>New York — wildposting / wheatpaste, print &amp; install</t>
+          <t>Philadelphia suburbs + New York</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Philadelphia; New York</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -10035,14 +10646,10 @@
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
+      <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr"/>
@@ -10050,7 +10657,7 @@
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://gsbdigital.com/</t>
+          <t>https://www.linkedin.com/company/catalyst-outdoor-advertising</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -10060,17 +10667,17 @@
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>Wildposting / production — quote only</t>
+          <t>Digital billboards — quote only</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
+          <t>Founded 2009 (Thaddeus Bartkowski); ~14 digital faces, known for 'living wall' displays. NOTE: financial distress in 2024; assets reportedly being sold to Lamar &amp; Clear Channel — verify current ownership before contacting.</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>gsbdigital.com; WebSearch 2026-07-08</t>
+          <t>Billboard Insider; Philadelphia Inquirer; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
@@ -10082,7 +10689,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Heritage Outdoor Media</t>
+          <t>GSB Digital</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -10092,7 +10699,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>New York (Times Square digital)</t>
+          <t>New York — wildposting / wheatpaste, print &amp; install</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -10119,7 +10726,11 @@
       <c r="I27" s="5" t="inlineStr"/>
       <c r="J27" s="5" t="inlineStr"/>
       <c r="K27" s="5" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>https://gsbdigital.com/</t>
+        </is>
+      </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -10127,17 +10738,17 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Times Square digital — quote only</t>
+          <t>Wildposting / production — quote only</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t>Times Square LED billboard technology.</t>
+          <t>Street-level wheatpaste/wildposting (SoHo, Williamsburg, LES, Bushwick, Harlem) + OOH production &amp; install.</t>
         </is>
       </c>
       <c r="P27" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>gsbdigital.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
@@ -10149,7 +10760,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Neutron Media</t>
+          <t>Heritage Outdoor Media</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -10159,7 +10770,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>New York (digital billboards)</t>
+          <t>New York (Times Square digital)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -10194,12 +10805,12 @@
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Times Square digital — quote only</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>Digital billboards in NYC's busiest corridors.</t>
+          <t>Times Square LED billboard technology.</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
@@ -10216,17 +10827,17 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Pearl Media</t>
+          <t>Neutron Media</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>New York / Times Square + experiential</t>
+          <t>New York (digital billboards)</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -10253,11 +10864,7 @@
       <c r="I29" s="5" t="inlineStr"/>
       <c r="J29" s="5" t="inlineStr"/>
       <c r="K29" s="5" t="inlineStr"/>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>https://pearlmedia.com/</t>
-        </is>
-      </c>
+      <c r="L29" s="5" t="inlineStr"/>
       <c r="M29" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -10265,17 +10872,17 @@
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Times Square / experiential — quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>Times Square billboards and experiential activations.</t>
+          <t>Digital billboards in NYC's busiest corridors.</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>pearlmedia.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
@@ -10287,17 +10894,17 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Red Rock Outdoor Advertising</t>
+          <t>Pearl Media</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>New York (Manhattan)</t>
+          <t>New York / Times Square + experiential</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -10324,7 +10931,11 @@
       <c r="I30" s="5" t="inlineStr"/>
       <c r="J30" s="5" t="inlineStr"/>
       <c r="K30" s="5" t="inlineStr"/>
-      <c r="L30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>https://pearlmedia.com/</t>
+        </is>
+      </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -10332,17 +10943,17 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Times Square / experiential — quote only</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Times Square billboards and experiential activations.</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>pearlmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -10354,17 +10965,17 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Rolling Adz Mobile Billboards</t>
+          <t>Red Rock Outdoor Advertising</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>New York City (mobile)</t>
+          <t>New York (Manhattan)</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -10391,11 +11002,7 @@
       <c r="I31" s="5" t="inlineStr"/>
       <c r="J31" s="5" t="inlineStr"/>
       <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr">
-        <is>
-          <t>https://rollingadz.com/</t>
-        </is>
-      </c>
+      <c r="L31" s="5" t="inlineStr"/>
       <c r="M31" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -10403,17 +11010,17 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard — day/route rate, quote only</t>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard fleet across NYC.</t>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>rollingadz.com; WebSearch 2026-07-08</t>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
@@ -10425,17 +11032,17 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Seen Outdoor Media, LLC</t>
+          <t>Rolling Adz Mobile Billboards</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>New York (Brooklyn)</t>
+          <t>New York City (mobile)</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -10451,7 +11058,7 @@
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Brooklyn</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -10462,7 +11069,11 @@
       <c r="I32" s="5" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="5" t="inlineStr"/>
-      <c r="L32" s="5" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>https://rollingadz.com/</t>
+        </is>
+      </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -10470,17 +11081,17 @@
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+          <t>Mobile billboard — day/route rate, quote only</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+          <t>Mobile billboard fleet across NYC.</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+          <t>rollingadz.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
@@ -10492,7 +11103,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>TSX Broadway (TSX Entertainment)</t>
+          <t>Seen Outdoor Media, LLC</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -10502,7 +11113,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Times Square (single landmark asset)</t>
+          <t>New York (Brooklyn)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -10518,7 +11129,7 @@
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Brooklyn</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -10537,27 +11148,94 @@
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr">
+        <is>
+          <t>On the NYC DOB Active Outdoor Advertising Companies (OAC) registry.</t>
+        </is>
+      </c>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>NYC DOB Active OAC list; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>TSX Broadway (TSX Entertainment)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Times Square (single landmark asset)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr"/>
+      <c r="K34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr"/>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
           <t>Premium spectacular — quote only, very high-end</t>
         </is>
       </c>
-      <c r="O33" s="5" t="inlineStr">
+      <c r="O34" s="5" t="inlineStr">
         <is>
           <t>Flagship 18k-sq-ft curved LED at 47th &amp; Broadway, Times Square.</t>
         </is>
       </c>
-      <c r="P33" s="5" t="inlineStr">
+      <c r="P34" s="5" t="inlineStr">
         <is>
           <t>WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q33" s="5" t="inlineStr">
+      <c r="Q34" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q33"/>
+  <autoFilter ref="A4:Q34"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -11836,12 +12514,12 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Los Angeles &amp; San Diego counties (SoCal)</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Los Angeles; San Diego</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -11861,7 +12539,7 @@
       <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>https://brayoutdoor.com/los-angeles-county/los-angeles-billboards/</t>
+          <t>https://brayoutdoor.com/</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
@@ -11876,7 +12554,7 @@
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
-          <t>LA-county billboard operator/agency.</t>
+          <t>SoCal billboard operator/media buyer across LA and San Diego counties.</t>
         </is>
       </c>
       <c r="P21" s="5" t="inlineStr">
@@ -14889,7 +15567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -14921,7 +15599,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>10 companies serving Phoenix · prices quote-only</t>
+          <t>11 companies serving Phoenix · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -15575,7 +16253,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Arizona Billboard Company</t>
+          <t>American Outdoor Advertising</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -15585,12 +16263,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Phoenix / Arizona</t>
+          <t>San Diego; Phoenix</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>San Diego; Phoenix</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -15599,14 +16277,10 @@
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Phoenix</t>
-        </is>
-      </c>
+      <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
@@ -15614,7 +16288,7 @@
       <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://arizonabillboardcompany.com/</t>
+          <t>https://www.americanoutdoor.com/</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -15629,12 +16303,12 @@
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>30+ yrs; billboards, digital LED, buses, shelters, airports, stadiums.</t>
+          <t>Digital &amp; static billboards on high-traffic routes; regional operator in San Diego and Phoenix.</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>arizonabillboardcompany.com; WebSearch 2026-07-08</t>
+          <t>americanoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q13" s="5" t="inlineStr">
@@ -15646,22 +16320,22 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>BM Outdoor Media</t>
+          <t>Arizona Billboard Company</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Independent / local operator</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>44 Texas cities + Phoenix</t>
+          <t>Phoenix / Arizona</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Houston; Dallas; San Antonio; Phoenix</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -15670,10 +16344,14 @@
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
@@ -15681,37 +16359,104 @@
       <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="5" t="inlineStr">
         <is>
+          <t>https://arizonabillboardcompany.com/</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>30+ yrs; billboards, digital LED, buses, shelters, airports, stadiums.</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>arizonabillboardcompany.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BM Outdoor Media</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>44 Texas cities + Phoenix</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Houston; Dallas; San Antonio; Phoenix</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
           <t>https://bmoutdoor.com/</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
-        <is>
-          <t>Quote only — request from company</t>
-        </is>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>Billboards, digital, transit &amp; street furniture across 44 TX cities and Phoenix.</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="P15" s="5" t="inlineStr">
         <is>
           <t>bmoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q14" s="5" t="inlineStr">
+      <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q14"/>
+  <autoFilter ref="A4:Q15"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -15726,7 +16471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -15758,7 +16503,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>10 companies serving Philadelphia · prices quote-only</t>
+          <t>13 companies serving Philadelphia · prices quote-only</t>
         </is>
       </c>
     </row>
@@ -16543,8 +17288,213 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Big Outdoor</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>New York; Philadelphia (digital spectaculars)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>New York; Philadelphia</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>https://bigoutdoor.com/</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Digital spectacular — quote only</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboard / spectacular operator (NYC + Philadelphia).</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Catalyst Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Philadelphia suburbs + New York</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Philadelphia; New York</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/catalyst-outdoor-advertising</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Digital billboards — quote only</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Founded 2009 (Thaddeus Bartkowski); ~14 digital faces, known for 'living wall' displays. NOTE: financial distress in 2024; assets reportedly being sold to Lamar &amp; Clear Channel — verify current ownership before contacting.</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Billboard Insider; Philadelphia Inquirer; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Keystone Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Philadelphia / Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Philadelphia</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.keystoneoutdoor.com/</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Static ~$1k–$25k+/4wk; premium/spectacular boards much higher (market avg)</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Regional PA billboard operator serving the Philadelphia market.</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q14"/>
+  <autoFilter ref="A4:Q17"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>

</xml_diff>